<commit_message>
update datumů šablon na 2025
</commit_message>
<xml_diff>
--- a/data/CMPA_template_cz.xlsx
+++ b/data/CMPA_template_cz.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\horkyt\Desktop\CMPA vzory\Completion rate předěláno na Kvalita zásahu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\horkyt\Desktop\repos\news-web2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA3DBEC-CA7E-4A80-9F00-7D33D3354C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF4FB74-0F98-4782-BBE5-4425D0AE77B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19005" yWindow="960" windowWidth="17475" windowHeight="17985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6375" yWindow="4395" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spoty" sheetId="2" r:id="rId1"/>
@@ -1641,7 +1641,7 @@
         <v>30</v>
       </c>
       <c r="F3" s="6">
-        <v>45127</v>
+        <v>45858</v>
       </c>
       <c r="H3" s="3">
         <v>0.81254629629629627</v>
@@ -1662,7 +1662,7 @@
         <v>30</v>
       </c>
       <c r="F4" s="6">
-        <v>45128</v>
+        <v>45859</v>
       </c>
       <c r="H4" s="3">
         <v>0.8125</v>
@@ -1683,7 +1683,7 @@
         <v>30</v>
       </c>
       <c r="F5" s="6">
-        <v>45129</v>
+        <v>45860</v>
       </c>
       <c r="H5" s="3">
         <v>0.8125</v>
@@ -1707,7 +1707,7 @@
         <v>30</v>
       </c>
       <c r="F6" s="6">
-        <v>45127</v>
+        <v>45858</v>
       </c>
       <c r="H6" s="3">
         <v>0.33320601851851855</v>
@@ -1731,7 +1731,7 @@
         <v>30</v>
       </c>
       <c r="F7" s="6">
-        <v>45128</v>
+        <v>45859</v>
       </c>
       <c r="H7" s="3">
         <v>0.33320601851851855</v>
@@ -1755,7 +1755,7 @@
         <v>30</v>
       </c>
       <c r="F8" s="6">
-        <v>45130</v>
+        <v>45861</v>
       </c>
       <c r="H8" s="3">
         <v>0.85416666666666696</v>
@@ -1776,7 +1776,7 @@
         <v>49</v>
       </c>
       <c r="F9" s="6">
-        <v>45126</v>
+        <v>45857</v>
       </c>
       <c r="J9">
         <v>150000</v>
@@ -1793,7 +1793,7 @@
         <v>51</v>
       </c>
       <c r="F10" s="6">
-        <v>45127</v>
+        <v>45858</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
@@ -1807,7 +1807,7 @@
         <v>52</v>
       </c>
       <c r="F11" s="6">
-        <v>45129</v>
+        <v>45860</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
@@ -1821,10 +1821,10 @@
         <v>28</v>
       </c>
       <c r="F12" s="6">
-        <v>45119</v>
+        <v>45850</v>
       </c>
       <c r="G12" s="6">
-        <v>45127</v>
+        <v>45858</v>
       </c>
       <c r="K12">
         <v>20000</v>
@@ -1859,10 +1859,10 @@
         <v>54</v>
       </c>
       <c r="F13" s="6">
-        <v>45110</v>
+        <v>45841</v>
       </c>
       <c r="G13" s="6">
-        <v>45110</v>
+        <v>45841</v>
       </c>
       <c r="K13">
         <v>15000</v>
@@ -1891,10 +1891,10 @@
         <v>70</v>
       </c>
       <c r="F14" s="6">
-        <v>45127</v>
+        <v>45858</v>
       </c>
       <c r="G14" s="6">
-        <v>45129</v>
+        <v>45860</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -1916,10 +1916,10 @@
         <v>57</v>
       </c>
       <c r="F15" s="6">
-        <v>45116</v>
+        <v>45847</v>
       </c>
       <c r="G15" s="6">
-        <v>45119</v>
+        <v>45850</v>
       </c>
       <c r="J15">
         <v>5000</v>
@@ -1942,10 +1942,10 @@
         <v>59</v>
       </c>
       <c r="F16" s="6">
-        <v>45116</v>
+        <v>45847</v>
       </c>
       <c r="G16" s="6">
-        <v>45119</v>
+        <v>45850</v>
       </c>
       <c r="M16">
         <v>50.226199999999999</v>
@@ -1962,10 +1962,10 @@
         <v>58</v>
       </c>
       <c r="F17" s="6">
-        <v>45116</v>
+        <v>45847</v>
       </c>
       <c r="G17" s="6">
-        <v>45119</v>
+        <v>45850</v>
       </c>
       <c r="M17">
         <v>50.226089999999999</v>
@@ -1985,10 +1985,10 @@
         <v>240</v>
       </c>
       <c r="F18" s="6">
-        <v>45116</v>
+        <v>45847</v>
       </c>
       <c r="G18" s="6">
-        <v>45119</v>
+        <v>45850</v>
       </c>
       <c r="M18">
         <v>50.088129500000001</v>

</xml_diff>